<commit_message>
S109: six map rows to green, three of them already were.
Four one-line repoints (281e8bd8) and the dispatch write (f4c98e91) on
both boxes, plus Trace_ProductHeaderView down to two divisions on each
box (JR20). Three further rows were already correct and the S108 survey
had recorded them wrong, so Step 1 was five real sites, not nine. The
bible reads 28 green, 16 red, 4 review of 48. Step 3's precondition is
built: 474 MO-0005 has two unequal receipts, without which row 31 cannot
be told from its own bug.
</commit_message>
<xml_diff>
--- a/UNITS-BIBLE.xlsx
+++ b/UNITS-BIBLE.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,15 +31,15 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
       <sz val="10"/>
     </font>
     <font>
@@ -60,11 +60,6 @@
       <color rgb="009C6500"/>
       <sz val="11"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -75,22 +70,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002F4F6F"/>
+        <fgColor rgb="001F3864"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00B7DFB7"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F4B6B6"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFE699"/>
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -120,19 +115,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -146,22 +138,16 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -530,9 +516,9 @@
   <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
@@ -997,16 +983,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1070,12 +1056,12 @@
           <t>3 STOCK ON HAND</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G2" s="6" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -1105,12 +1091,12 @@
           <t>4 PRD-TO-DATE</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -1140,12 +1126,12 @@
           <t>Dispatch</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -1175,12 +1161,12 @@
           <t>4 PRD-TO-DATE</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -1210,12 +1196,12 @@
           <t>Dispatch / 4</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -1245,12 +1231,12 @@
           <t>4 PRD-TO-DATE</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -1280,12 +1266,12 @@
           <t>1 ING-REQ</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -1315,12 +1301,12 @@
           <t>1 ING-REQ</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -1350,12 +1336,12 @@
           <t>1 ING-REQ</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -1385,12 +1371,12 @@
           <t>1 ING-REQ</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="G11" s="5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -1420,12 +1406,12 @@
           <t>1 ING-REQ</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="G12" s="5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -1455,12 +1441,12 @@
           <t>4 PRD-TO-DATE</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr">
+      <c r="G13" s="5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -1490,12 +1476,12 @@
           <t>Dispatch</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -1525,12 +1511,12 @@
           <t>Dispatch</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -1560,12 +1546,12 @@
           <t>Dispatch</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G16" s="6" t="inlineStr">
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -1595,12 +1581,12 @@
           <t>Dispatch</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="F17" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
+      <c r="G17" s="5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -1630,12 +1616,12 @@
           <t>Dispatch</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G18" s="6" t="inlineStr">
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -1665,12 +1651,12 @@
           <t>2 PK-CASCADE</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr">
+      <c r="G19" s="5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -1700,12 +1686,12 @@
           <t>2 PK-CASCADE</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr">
+      <c r="G20" s="5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -1735,14 +1721,14 @@
           <t>defect</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
-        <is>
-          <t>Step 1</t>
-        </is>
-      </c>
-      <c r="G21" s="7" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Step 6</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
     </row>
@@ -1757,12 +1743,12 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>rejected-materials.ts:154</t>
+          <t>rejected-materials.html:63</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>qty_rejected / weight</t>
+          <t>qty_rejected_units, type-gated. WAS ALREADY OK — the survey named the wrong line</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
@@ -1770,14 +1756,14 @@
           <t>4 PRD-TO-DATE</t>
         </is>
       </c>
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t>Step 2</t>
-        </is>
-      </c>
-      <c r="G22" s="7" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>— (survey error)</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
     </row>
@@ -1797,7 +1783,7 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>received_qty / weight</t>
+          <t>received_units</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
@@ -1805,14 +1791,14 @@
           <t>4 PRD-TO-DATE</t>
         </is>
       </c>
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t>Step 2</t>
-        </is>
-      </c>
-      <c r="G23" s="7" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>S109 proven</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
     </row>
@@ -1832,7 +1818,7 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>received_qty / weight</t>
+          <t>received_units. DEPLOYED, NOT SCREEN-PROVEN</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
@@ -1840,14 +1826,14 @@
           <t>4 PRD-TO-DATE</t>
         </is>
       </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>Step 2</t>
-        </is>
-      </c>
-      <c r="G24" s="7" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>S109 unproven</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
     </row>
@@ -1867,7 +1853,7 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>received_qty / weight</t>
+          <t>received_units</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
@@ -1875,14 +1861,14 @@
           <t>4 PRD-TO-DATE</t>
         </is>
       </c>
-      <c r="F25" s="5" t="inlineStr">
-        <is>
-          <t>Step 2</t>
-        </is>
-      </c>
-      <c r="G25" s="7" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>S109 proven</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
     </row>
@@ -1902,7 +1888,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>getWdu on received_qty</t>
+          <t>getWdu on received_qty. NOT a repoint — the helper divides</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
@@ -1910,14 +1896,14 @@
           <t>4 PRD-TO-DATE</t>
         </is>
       </c>
-      <c r="F26" s="5" t="inlineStr">
-        <is>
-          <t>Step 2</t>
-        </is>
-      </c>
-      <c r="G26" s="7" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>row 46 sitting</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
     </row>
@@ -1932,12 +1918,12 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>product-traceability.ts:109</t>
+          <t>product-traceability.ts:113</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>received_qty / weight</t>
+          <t>received_units. WAS ALREADY OK — carries its own comment</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
@@ -1945,14 +1931,14 @@
           <t>4 PRD-TO-DATE</t>
         </is>
       </c>
-      <c r="F27" s="5" t="inlineStr">
-        <is>
-          <t>Step 2</t>
-        </is>
-      </c>
-      <c r="G27" s="7" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>— (survey error)</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
     </row>
@@ -1972,7 +1958,7 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>inventory / weight</t>
+          <t>inventory_units, x weight at :885. WAS ALREADY OK</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
@@ -1980,14 +1966,14 @@
           <t>3 STOCK ON HAND</t>
         </is>
       </c>
-      <c r="F28" s="5" t="inlineStr">
-        <is>
-          <t>Step 2</t>
-        </is>
-      </c>
-      <c r="G28" s="7" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>— (survey error)</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
     </row>
@@ -2007,7 +1993,7 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>(inventory/batch) x (batch/weight)</t>
+          <t>inventory_units. Kg half left reading inventory by design</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
@@ -2015,14 +2001,14 @@
           <t>3 STOCK ON HAND</t>
         </is>
       </c>
-      <c r="F29" s="5" t="inlineStr">
-        <is>
-          <t>Step 2</t>
-        </is>
-      </c>
-      <c r="G29" s="7" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>S109 proven</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
     </row>
@@ -2042,7 +2028,7 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>qty_rejected / weight</t>
+          <t>rmp.qty_rejected_units, CTE type-gated to Product. BOTH BOXES</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
@@ -2050,14 +2036,14 @@
           <t>4 PRD-TO-DATE</t>
         </is>
       </c>
-      <c r="F30" s="5" t="inlineStr">
-        <is>
-          <t>Step 2</t>
-        </is>
-      </c>
-      <c r="G30" s="7" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>S109 proven</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
     </row>
@@ -2072,12 +2058,12 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>add-dispatch-v2.ts:194</t>
+          <t>add-dispatch-v2.ts:183,194</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>divides, rounds, STORES packing_units</t>
+          <t>sums the operator's TYPED qtyWdu. No division</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
@@ -2085,14 +2071,14 @@
           <t>2 PK-CASCADE</t>
         </is>
       </c>
-      <c r="F31" s="5" t="inlineStr">
-        <is>
-          <t>Step 3</t>
-        </is>
-      </c>
-      <c r="G31" s="7" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>S109 proven</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
     </row>
@@ -2120,14 +2106,14 @@
           <t>4 PRD-TO-DATE</t>
         </is>
       </c>
-      <c r="F32" s="5" t="inlineStr">
-        <is>
-          <t>Step 4a</t>
-        </is>
-      </c>
-      <c r="G32" s="7" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>Step 3a</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
     </row>
@@ -2155,14 +2141,14 @@
           <t>1 ING-REQ</t>
         </is>
       </c>
-      <c r="F33" s="5" t="inlineStr">
-        <is>
-          <t>Step 4b</t>
-        </is>
-      </c>
-      <c r="G33" s="7" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>Step 3b</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
     </row>
@@ -2190,14 +2176,14 @@
           <t>3 STOCK ON HAND</t>
         </is>
       </c>
-      <c r="F34" s="5" t="inlineStr">
-        <is>
-          <t>Step 4c</t>
-        </is>
-      </c>
-      <c r="G34" s="7" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>Step 3c</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
     </row>
@@ -2225,14 +2211,14 @@
           <t>1 ING-REQ</t>
         </is>
       </c>
-      <c r="F35" s="5" t="inlineStr">
-        <is>
-          <t>Step 4d</t>
-        </is>
-      </c>
-      <c r="G35" s="7" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>Step 3d</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
     </row>
@@ -2260,14 +2246,14 @@
           <t>1 ING-REQ</t>
         </is>
       </c>
-      <c r="F36" s="5" t="inlineStr">
-        <is>
-          <t>Step 5</t>
-        </is>
-      </c>
-      <c r="G36" s="7" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>Step 4</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
     </row>
@@ -2295,14 +2281,14 @@
           <t>1 ING-REQ</t>
         </is>
       </c>
-      <c r="F37" s="5" t="inlineStr">
-        <is>
-          <t>Step 5</t>
-        </is>
-      </c>
-      <c r="G37" s="7" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>Step 4</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
     </row>
@@ -2327,17 +2313,17 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>1 ING-REQ</t>
-        </is>
-      </c>
-      <c r="F38" s="5" t="inlineStr">
-        <is>
-          <t>Step 6</t>
-        </is>
-      </c>
-      <c r="G38" s="7" t="inlineStr">
-        <is>
-          <t>✗</t>
+          <t>3 STOCK ON HAND</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>Step 5</t>
+        </is>
+      </c>
+      <c r="G38" s="6" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
     </row>
@@ -2357,7 +2343,7 @@
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>subtracts Kg terms, then divides</t>
+          <t>five Kg terms, then divides</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
@@ -2365,14 +2351,14 @@
           <t>3 STOCK ON HAND</t>
         </is>
       </c>
-      <c r="F39" s="5" t="inlineStr">
-        <is>
-          <t>Step 6</t>
-        </is>
-      </c>
-      <c r="G39" s="7" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>Step 5</t>
+        </is>
+      </c>
+      <c r="G39" s="6" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
     </row>
@@ -2382,7 +2368,7 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>IP trace — backward</t>
+          <t>IP trace backward</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
@@ -2392,22 +2378,22 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>qty_allocated / weight</t>
+          <t>qty_allocated / weight, no whd_flag filter</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>1 ING-REQ</t>
-        </is>
-      </c>
-      <c r="F40" s="5" t="inlineStr">
-        <is>
-          <t>Step 6</t>
-        </is>
-      </c>
-      <c r="G40" s="7" t="inlineStr">
-        <is>
-          <t>✗</t>
+          <t>3 STOCK ON HAND</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>Step 5</t>
+        </is>
+      </c>
+      <c r="G40" s="6" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
     </row>
@@ -2417,7 +2403,7 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>IP trace — forward</t>
+          <t>IP trace forward</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -2432,17 +2418,17 @@
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>1 ING-REQ</t>
-        </is>
-      </c>
-      <c r="F41" s="5" t="inlineStr">
-        <is>
-          <t>Step 6</t>
-        </is>
-      </c>
-      <c r="G41" s="7" t="inlineStr">
-        <is>
-          <t>✗</t>
+          <t>3 STOCK ON HAND</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>Step 5</t>
+        </is>
+      </c>
+      <c r="G41" s="6" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
     </row>
@@ -2462,22 +2448,22 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>serves Kg only, no unit figure</t>
+          <t>no unit column exists yet</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>1 ING-REQ</t>
-        </is>
-      </c>
-      <c r="F42" s="5" t="inlineStr">
-        <is>
-          <t>Step 6</t>
-        </is>
-      </c>
-      <c r="G42" s="7" t="inlineStr">
-        <is>
-          <t>✗</t>
+          <t>3 STOCK ON HAND</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>Step 5</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
     </row>
@@ -2497,22 +2483,22 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>serves Kg only, no unit figure</t>
+          <t>no unit column exists yet</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>1 ING-REQ</t>
-        </is>
-      </c>
-      <c r="F43" s="5" t="inlineStr">
-        <is>
-          <t>Step 7</t>
-        </is>
-      </c>
-      <c r="G43" s="7" t="inlineStr">
-        <is>
-          <t>✗</t>
+          <t>3 STOCK ON HAND</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>Step 6</t>
+        </is>
+      </c>
+      <c r="G43" s="6" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2508,7 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>Product return — stock balance</t>
+          <t>Product return stock balance</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
@@ -2532,7 +2518,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>adds back to Kg only</t>
+          <t>adds Kg back, never touches inventory_units</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
@@ -2540,14 +2526,14 @@
           <t>3 STOCK ON HAND</t>
         </is>
       </c>
-      <c r="F44" s="5" t="inlineStr">
-        <is>
-          <t>Step 7</t>
-        </is>
-      </c>
-      <c r="G44" s="7" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>Step 6</t>
+        </is>
+      </c>
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
     </row>
@@ -2572,15 +2558,15 @@
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>MISLABEL</t>
-        </is>
-      </c>
-      <c r="F45" s="5" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="G45" s="8" t="inlineStr">
+          <t>Dispatch</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="G45" s="7" t="inlineStr">
         <is>
           <t>?</t>
         </is>
@@ -2602,20 +2588,20 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>qty / weight — materials are Kg by design</t>
+          <t>Kg-anchored, may be correct by design</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F46" s="5" t="inlineStr">
-        <is>
-          <t>Verify</t>
-        </is>
-      </c>
-      <c r="G46" s="8" t="inlineStr">
+          <t>3 STOCK ON HAND</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="G46" s="7" t="inlineStr">
         <is>
           <t>?</t>
         </is>
@@ -2637,20 +2623,20 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>callers pass DIFFERENT sources</t>
+          <t>some callers pass Kg and are CORRECT</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>MIXED</t>
-        </is>
-      </c>
-      <c r="F47" s="5" t="inlineStr">
-        <is>
-          <t>Own sitting</t>
-        </is>
-      </c>
-      <c r="G47" s="8" t="inlineStr">
+          <t>4 PRD-TO-DATE</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>own sitting</t>
+        </is>
+      </c>
+      <c r="G47" s="7" t="inlineStr">
         <is>
           <t>?</t>
         </is>
@@ -2677,17 +2663,52 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F48" s="5" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
-      <c r="G48" s="8" t="inlineStr">
+          <t>Dispatch</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>delete</t>
+        </is>
+      </c>
+      <c r="G48" s="7" t="inlineStr">
         <is>
           <t>?</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Stock popup — MO card labels</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>formulation-edit-stock-info</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>15.170 (41.000 Kg) — Kg and units TRANSPOSED. NEW S109</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>3 STOCK ON HAND</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>unfiled</t>
+        </is>
+      </c>
+      <c r="G49" s="6" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
     </row>
@@ -2702,12 +2723,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
@@ -2748,12 +2769,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Today</t>
+          <t>S108</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>19 sites already follow the rule</t>
+          <t>As the survey recorded it</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -2761,284 +2782,452 @@
           <t>—</t>
         </is>
       </c>
-      <c r="D2" s="9" t="n">
+      <c r="D2" s="8" t="n">
         <v>19</v>
       </c>
-      <c r="E2" s="10" t="n">
+      <c r="E2" s="9" t="n">
         <v>24</v>
       </c>
-      <c r="F2" s="11" t="n">
+      <c r="F2" s="10" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Step 1</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>The returnSum bug. Live on both clients</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>#20</t>
-        </is>
-      </c>
-      <c r="D3" s="9" t="n">
-        <v>20</v>
-      </c>
-      <c r="E3" s="10" t="n">
-        <v>23</v>
-      </c>
-      <c r="F3" s="11" t="n">
+          <t>Corrected</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Rows 21, 26 and 27 were ALREADY green</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>#21 #26 #27</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="n">
+        <v>22</v>
+      </c>
+      <c r="E3" s="9" t="n">
+        <v>21</v>
+      </c>
+      <c r="F3" s="10" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Step 2</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Nine one-line repoints, one build</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>#21 #22 #23 #24 #25 #26 #27 #28 #29</t>
-        </is>
-      </c>
-      <c r="D4" s="9" t="n">
-        <v>29</v>
-      </c>
-      <c r="E4" s="10" t="n">
-        <v>14</v>
-      </c>
-      <c r="F4" s="11" t="n">
+          <t>S109 a</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Four repoints, one build. Commit 281e8bd8</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>#22 #23 #24 #28</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="n">
+        <v>26</v>
+      </c>
+      <c r="E4" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="F4" s="10" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Step 3</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>The dispatch write path</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>#30</t>
-        </is>
-      </c>
-      <c r="D5" s="9" t="n">
-        <v>30</v>
-      </c>
-      <c r="E5" s="10" t="n">
-        <v>13</v>
-      </c>
-      <c r="F5" s="11" t="n">
+          <t>+ row 48</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>New site found while verifying</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>26</v>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="F5" s="10" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Step 4</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Four procedure changes</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>#31 #32 #33 #34</t>
-        </is>
-      </c>
-      <c r="D6" s="9" t="n">
-        <v>34</v>
-      </c>
-      <c r="E6" s="10" t="n">
-        <v>9</v>
-      </c>
-      <c r="F6" s="11" t="n">
+          <t>S109 b</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>The dispatch write. Commit f4c98e91</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>#30</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>27</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="F6" s="10" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Step 5</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>The requirement calculation</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>#35 #36</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="n">
-        <v>36</v>
-      </c>
-      <c r="E7" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="F7" s="11" t="n">
+          <t>S109 c</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>The view, misc release. BOTH BOXES</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>#29</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>28</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="F7" s="10" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Step 6</t>
+          <t>Step 3</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>The schema — P82 CLOSES HERE</t>
+          <t>Four procedure changes. NEEDS A MULTI-RECEIPT FIXTURE FIRST</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>#37 #38 #39 #40 #41</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="n">
-        <v>41</v>
-      </c>
-      <c r="E8" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="F8" s="11" t="n">
+          <t>#31 #32 #33 #34</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>32</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="F8" s="10" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Step 7</t>
+          <t>Step 4</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>The return path</t>
+          <t>The requirement calculation. Own session, own gate</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>#42 #43</t>
-        </is>
-      </c>
-      <c r="D9" s="9" t="n">
+          <t>#35 #36</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>34</v>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="F9" s="10" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Step 5</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>The schema — P82 CLOSES HERE</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>#37 #38 #39 #40 #41</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>39</v>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="F10" s="10" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Step 6</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>The return path — SURVEY FIRST, not a fix list</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>#20 #42 #43</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>42</v>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" s="10" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Row 46</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>The seven-copy helper, its own sitting</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>#25</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="n">
         <v>43</v>
       </c>
-      <c r="E9" s="10" t="n">
+      <c r="E12" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="10" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Row 48</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>The transposed labels</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>#48</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>44</v>
+      </c>
+      <c r="E13" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="F9" s="11" t="n">
+      <c r="F13" s="10" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="12" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>WHERE WE ARE</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>28 green, 16 red, 4 to review, out of 48. S109 moved six rows: four repoints, the dispatch write, and the view.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>NEXT TARGET — Step 3, four rows.</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>BUILD THE FIXTURE FIRST. 474 MO-0003 has ONE receipt, so per-receipt and MO-total coincide and a fix cannot be told from the bug. A second MO with TWO receipts is the precondition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>The four to review are not defects.</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>#44 a mislabelled field, #45 probably correct by design, #46 needs each caller read, #47 dead code.</t>
         </is>
       </c>
-      <c r="C11" s="14" t="inlineStr"/>
-      <c r="D11" s="14" t="inlineStr"/>
-      <c r="E11" s="14" t="inlineStr"/>
-      <c r="F11" s="14" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="13" t="inlineStr">
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>MO-0004 on company 474 is the test.</t>
         </is>
       </c>
-      <c r="B12" s="14" t="inlineStr">
-        <is>
-          <t>Do not release it. It is the before picture.</t>
-        </is>
-      </c>
-      <c r="C12" s="14" t="inlineStr"/>
-      <c r="D12" s="14" t="inlineStr"/>
-      <c r="E12" s="14" t="inlineStr"/>
-      <c r="F12" s="14" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Do not release it. It is the before picture for Step 4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Pouch 4347.000 Ea is the control.</t>
         </is>
       </c>
-      <c r="B13" s="14" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>It must NOT move at any step. If it does, the fix is wrong.</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr"/>
-      <c r="D13" s="14" t="inlineStr"/>
-      <c r="E13" s="14" t="inlineStr"/>
-      <c r="F13" s="14" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="13" t="inlineStr">
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>#1 stock-info.ts:188 is the model.</t>
         </is>
       </c>
-      <c r="B14" s="14" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Read the stored count, multiply for the Kg. Do not invent a third shape.</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr"/>
-      <c r="D14" s="14" t="inlineStr"/>
-      <c r="E14" s="14" t="inlineStr"/>
-      <c r="F14" s="14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="13" t="inlineStr">
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>This is a living document.</t>
         </is>
       </c>
-      <c r="B15" s="14" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>Anything found later gets a row. It does not have to be complete to be useful.</t>
         </is>
       </c>
-      <c r="C15" s="14" t="inlineStr"/>
-      <c r="D15" s="14" t="inlineStr"/>
-      <c r="E15" s="14" t="inlineStr"/>
-      <c r="F15" s="14" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>S109 — the survey was wrong in BOTH directions.</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Three rows were marked red and were already green. #25 was listed as a one-line repoint and is not — it calls a helper that divides.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>S109 — #23 is green but unproven.</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Deployed to both boxes and never seen on a screen; /MLO-Management redirects under the test user's roles. Same line and procedure as #22 and #24, both proven. First item at the next open.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>S109 — #29 traded correct-derived for incomplete-stored.</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>On rows written BEFORE JR15 (S103) no unit count was ever stored, so those cells now read 0 or low. MEASURED: no client row is affected — Glutenull has no MR rows, Hagensborg's 24 are all Material with no mlc_id. Only sandbox 464 moved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>S109 — #30 is preventive on prod, not corrective.</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Neither client has ever created a dispatch order. All nine DOs on prod are sandbox, all on round ratios where the old division landed exactly. Nothing to heal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>The step numbers moved at the S108 close.</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>The return path became Step 6 and goes LAST. This sheet uses the current numbering, matching PLAN.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
S112 close: the Step 5 groundwork, a regression S111 caused and repaired, the composite display, and two rulings that decide the rest of the campaign. No row moved to green. Three rows added and row 45 rescoped, so the board reads 36 of 51 and the balance grew from 14 to 15. S113 is now the only wrong number in the queue - Material Traceability prints an MO's unit count as kilograms and then divides it, traced end to end through seven hops to a procedure in no bible row.
</commit_message>
<xml_diff>
--- a/UNITS-BIBLE.xlsx
+++ b/UNITS-BIBLE.xlsx
@@ -538,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E63"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -565,7 +565,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Updated at the close of S111, 9 August 2026.   BOARD: 34 GREEN · 0 PART · 10 RED · 4 REVIEW, of 48.</t>
+          <t>Updated at the close of S112, 10 August 2026.   BOARD: 36 GREEN · 0 PART · 12 RED · 3 REVIEW, of 51.</t>
         </is>
       </c>
     </row>
@@ -1632,24 +1632,24 @@
       <c r="A50" s="5" t="n">
         <v>45</v>
       </c>
-      <c r="B50" s="9" t="inlineStr">
-        <is>
-          <t>??</t>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>XX</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>Material traceability</t>
+          <t>Material traceability - A MIXED SCREEN</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>material-traceability-details:169,170</t>
+          <t>material-traceability-details.ts:169,170 + html :107 :108 :123 :124 :215 :216</t>
         </is>
       </c>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>Materials are Kg-anchored BY DESIGN, so this may be correct. VERIFY AGAINST THE RULE.</t>
+          <t>RE-SCOPED S112 AND NO LONGER A REVIEW ITEM. IT IS THE ONLY WRONG NUMBER IN THE QUEUE - MO-0010 reads 10 Kg (1#) where the truth is 100 Kg, 10 units, and the Completed figure on the SAME ROW reads 100 Kg (10#) and is correct. CAUSE: mlomanagement.qty holds UNITS since the S41 flip; this screen prints it with a Kg label AND divides it by wgt_kgs_per_unit. Its neighbour received_qty really is Kg, so half the row kept working and nobody noticed. Traced end to end 10 Aug, seven hops, to Trace_MaterialDetails_SP - WHICH IS IN NO BIBLE ROW, see row 51. The procedure is INNOCENT; the defect is entirely frontend. The MATERIAL rows at :107/:108 are FINE - that alarm was withdrawn. -&gt; S113.</t>
         </is>
       </c>
     </row>
@@ -1749,74 +1749,124 @@
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>NEW — FOUND S111, IN NO PRIOR ROW. Read the Kg inventory column one block below a corrected figure. Fixed in the same session: reads inventory_units. The matList line beside it reads the SAME property and is CORRECT — materials are Kg-anchored by rule. NEEDS MINTY'S RULING on whether it stands as a row.</t>
+          <t>ADDED S111, ACCEPTED AS ITS OWN ROW BY MINTY IN S112. Read the Kg inventory column one block below a corrected figure. Fixed in the same session: reads inventory_units. The matList line beside it reads the SAME property and is CORRECT — materials are Kg-anchored by rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="n">
+        <v>51</v>
+      </c>
+      <c r="B55" s="10" t="inlineStr">
+        <is>
+          <t>XX</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>Trace_MaterialDetails_SP - IN NO PRIOR ROW</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>api/models/Traceability.js:360</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="inlineStr">
+        <is>
+          <t>FOUND S112 by tracing row 45's defect to its source. It feeds the WHOLE Material Traceability screen and the survey never mapped it - rows 37-41 name five procedures and this is a SIXTH. It is INNOCENT: it hands over mlomanagement.qty (units) and mlomanagement.received_qty (Kg) honestly and does no arithmetic. It is listed RED only because it must gain mlomanagement.received_units for row 45's fix. -&gt; S113, and it is the fourth unmapped site found in S112.</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="3" t="inlineStr">
+      <c r="A56" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="B56" s="10" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>Release screen - the PRODUCT block</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>release-mat-details html :115 :125 :157 :158 + ts :296</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="inlineStr">
+        <is>
+          <t>ADDED S112, AND ADDED BECAUSE S111 BROKE IT. S111 made final_qty a UNIT count for the MO detail screens; this screen reads the same property and pairs it with KILOGRAM inputs, so the auto-fill put 4.846 units into a Kg box and the guard TURNED GREEN on a release of nearly THREE TIMES the requirement. Zero client exposure - neither client has intermediates. FIXED ADDITIVELY: the backend now serves final_qty_kg alongside final_qty and this screen reads the Kg one, so rows 34 and 36 stand. Green as a consistent Kg-anchored screen, and it stays green when S113 makes it units-anchored.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
         <is>
           <t>LEGEND</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="11" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="C57" s="12" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="C59" s="12" t="inlineStr">
         <is>
           <t>reads a stored count, follows the rule</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="13" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="13" t="inlineStr">
         <is>
           <t>XX</t>
         </is>
       </c>
-      <c r="C58" s="12" t="inlineStr">
+      <c r="C60" s="12" t="inlineStr">
         <is>
           <t>calculates instead</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="14" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="14" t="inlineStr">
         <is>
           <t>??</t>
         </is>
       </c>
-      <c r="C59" s="12" t="inlineStr">
+      <c r="C61" s="12" t="inlineStr">
         <is>
           <t>to review, not a defect</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="15" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="15" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
-      <c r="C60" s="12" t="inlineStr">
-        <is>
-          <t>row 49 — found S111, needs Minty's ruling on whether it stands as a row</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="3" t="inlineStr">
+      <c r="C62" s="12" t="inlineStr">
+        <is>
+          <t>rows 49, 50 and 51 — added S111 and S112</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
         <is>
           <t>A ROW IS GREEN WHEN IT SATISFIES PART 1, NOT WHEN IT WAS TOUCHED. A MOVING NUMBER IS NOT PROOF OF A CLOSED ROW.</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="3" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
         <is>
           <t>AN ADDRESS IS A CLAIM. S111 corrected SIX of them (rows 19, 34, 35, 36 and two frontend sites). READ THE LINE BEFORE PATCHING IT.</t>
         </is>
@@ -1833,7 +1883,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1855,7 +1905,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>44 IS THE CEILING, NOT 48. Rows 44, 45, 46 and 47 are REVIEW items — they close as DECISIONS, not fixes. If row 49 is accepted, the ceiling becomes 45 of 49.</t>
+          <t>47 IS THE CEILING, OF 51. Rows 44, 46 and 47 close as DECISIONS. Row 45 is NO LONGER one of them - it is the only WRONG NUMBER in the queue and it is S113.</t>
         </is>
       </c>
     </row>
@@ -2005,121 +2055,129 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>S111</t>
         </is>
       </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>rows 32, 33, 34, 36 — the intermediate basis</t>
         </is>
       </c>
-      <c r="C9" s="6" t="n">
+      <c r="C9" s="5" t="n">
         <v>34</v>
       </c>
-      <c r="D9" s="6" t="n">
+      <c r="D9" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="6" t="n">
+      <c r="E9" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="F9" s="6" t="n">
+      <c r="F9" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="G9" s="6" t="n">
+      <c r="G9" s="5" t="n">
         <v>48</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>S111 close</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>row 49 accepted as its own row</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>49</v>
+      </c>
+    </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>S112</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>rows 50 and 51 added; row 45 rescoped to RED. NO ROW MOVED TO OK.</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>What it is</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Rows</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>Takes green to</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr"/>
-      <c r="F11" s="4" t="inlineStr"/>
-      <c r="G11" s="4" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>STEP 5</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>the schema — qty_allocated_units. P82's ARITHMETIC CLOSES HERE</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>37,38,39,40,41</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="n">
-        <v>39</v>
-      </c>
-      <c r="E12" s="7" t="inlineStr"/>
-      <c r="F12" s="7" t="inlineStr"/>
-      <c r="G12" s="7" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>STEP 6</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>the return path. SURVEY FIRST — P168's cause has never been read</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>20,42,43</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="n">
-        <v>42</v>
-      </c>
-      <c r="E13" s="7" t="inlineStr"/>
-      <c r="F13" s="7" t="inlineStr"/>
-      <c r="G13" s="7" t="inlineStr"/>
+      <c r="E13" s="4" t="inlineStr"/>
+      <c r="F13" s="4" t="inlineStr"/>
+      <c r="G13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>ROW 25</t>
+          <t>S113</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>the seven-copy helper, its own sitting</t>
+          <t>rows 45 and 51 - THE ONLY WRONG NUMBER IN THE QUEUE. Half a session</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>45,51</t>
         </is>
       </c>
       <c r="D14" s="5" t="n">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="E14" s="7" t="inlineStr"/>
       <c r="F14" s="7" t="inlineStr"/>
@@ -2128,21 +2186,21 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>ROW 48</t>
+          <t>S114</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>the transposed labels</t>
+          <t>THE UNITS CAPTURE on the release screen. MOVES NO ROW - it UNBLOCKS FIVE</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D15" s="5" t="n">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="E15" s="7" t="inlineStr"/>
       <c r="F15" s="7" t="inlineStr"/>
@@ -2151,30 +2209,106 @@
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>S115</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>rows 44/45/46/47 — decisions, not fixes</t>
+          <t>rows 37-41. P82's ARITHMETIC CLOSES. TRAPS 10 RETIRES</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>44,45,46,47</t>
+          <t>37,38,39,40,41</t>
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E16" s="7" t="inlineStr"/>
       <c r="F16" s="7" t="inlineStr"/>
       <c r="G16" s="7" t="inlineStr"/>
     </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>S116</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>rows 20/42/43, the return path. Minty's ruling S112: LAST</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>20,42,43</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="E17" s="7" t="inlineStr"/>
+      <c r="F17" s="7" t="inlineStr"/>
+      <c r="G17" s="7" t="inlineStr"/>
+    </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>S111's PRECONDITION WAS ALREADY MEASURED AND HELD: subrecipeformulation.ship_qty is populated on EVERY row of BOTH boxes — dev 15, prod 10, zero null or zero. NO HEAL WAS NEEDED.</t>
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>S117</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>row 25 and row 48, the tail. THE CEILING</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>25,48</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="E18" s="7" t="inlineStr"/>
+      <c r="F18" s="7" t="inlineStr"/>
+      <c r="G18" s="7" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>REVIEW</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>rows 44/46/47 — decisions, not fixes</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>44,46,47</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="E19" s="7" t="inlineStr"/>
+      <c r="F19" s="7" t="inlineStr"/>
+      <c r="G19" s="7" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>S114 CANNOT RUN BEFORE S113. The qty_allocated_units column exists on DEV and IS EMPTY. A read repointed against an unpopulated column shows 0 - worse than the division it replaces, because a plausible wrong number becomes an obviously wrong zero on a client-facing traceability screen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>MINTY'S RULING, S112: ANY INTERMEDIATE-PRODUCT FIGURE, ANYWHERE INCLUDING TRACEABILITY, SHOWS UNITS WITH Kg DERIVED BESIDE IT - units# (Kg uom). Units are the anchor end to end. This is why rows 37-41 get REPOINTED rather than excused as correct-by-design.</t>
         </is>
       </c>
     </row>
@@ -2573,7 +2707,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2681,17 +2815,34 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>S112</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>10 Aug 2026</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>NO ROW MOVED TO OK. Two rows added, both already green, so the balance is unchanged at 14. Row 49 ACCEPTED. Row 50 ADDED - the release screen's product block, BROKEN BY S111 and repaired in S112. TWO RULINGS BY MINTY: units are the anchor end to end including traceability, which decides Step 5; and materials are Kg only, which re-scoped row 45 from a review item to a job. PART 1 UNTOUCHED BY CLAUDE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>S111</t>
         </is>
       </c>
-      <c r="B9" s="21" t="inlineStr">
+      <c r="B10" s="21" t="inlineStr">
         <is>
           <t>9 Aug 2026</t>
         </is>
       </c>
-      <c r="C9" s="21" t="inlineStr">
+      <c r="C10" s="21" t="inlineStr">
         <is>
           <t>ROWS 32, 33, 34 AND 36 -&gt; OK. The PART status RETIRES — no row wears it. Both intermediate procedures now serve ship_qty and inventory_units. SIX ADDRESSES CORRECTED (rows 19, 34, 35, 36 and two frontend sites). ROW 49 ADDED — a Batch Materials stock site in no prior row, found and fixed the same session; NEEDS MINTY'S RULING on whether it stands. PART 1 UNTOUCHED.</t>
         </is>

</xml_diff>